<commit_message>
Refactor: decouple launcher from type, add sword/sword_qi ATK system, fix battle board init
- Launcher detection: field-based (spawns+max_charges) instead of type==LAUNCHER
- EffectType: add QI=6, ATK_BOOST=7; remove old SWORD_QI API
- Sword (type=4, effect_type=7): launcher that spawns sword qi with atk_base snapshot
- Sword qi merge: atk_base values sum; damage = atk_base × effect_value
- Battle board: fix stale grid cache, getInitialSetup ?? fallback, board_type-aware reinit
- GM panel: token-based sync, light sync for value-only commands, full sync for grid changes
- Config: load effect items (type=5) server-side, parse_ingredient_list strips count
- Rewards 1-10: exp (token=4) instead of stamina/spirit_stones

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/xlsx/items.xlsx
+++ b/config/xlsx/items.xlsx
@@ -6467,7 +6467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H211"/>
+  <dimension ref="A1:M211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6478,6 +6478,11 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6521,6 +6526,31 @@
           <t>effect_value</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>max_charges</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>recharge_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>no_cost</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>spawns(id:weight)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>fixed_spawns</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -6549,6 +6579,11 @@
       <c r="H2" s="3" t="n">
         <v>50</v>
       </c>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -6577,6 +6612,11 @@
       <c r="H3" s="3" t="n">
         <v>50</v>
       </c>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -6605,6 +6645,11 @@
       <c r="H4" s="3" t="n">
         <v>50</v>
       </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr"/>
+      <c r="M4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -6633,6 +6678,11 @@
       <c r="H5" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -6661,6 +6711,11 @@
       <c r="H6" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -6689,6 +6744,11 @@
       <c r="H7" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -6717,6 +6777,11 @@
       <c r="H8" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
+      <c r="M8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -6745,6 +6810,11 @@
       <c r="H9" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -6773,6 +6843,11 @@
       <c r="H10" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -6801,6 +6876,11 @@
       <c r="H11" s="3" t="n">
         <v>400</v>
       </c>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -6829,6 +6909,11 @@
       <c r="H12" s="3" t="n">
         <v>750</v>
       </c>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -6857,6 +6942,11 @@
       <c r="H13" s="3" t="n">
         <v>750</v>
       </c>
+      <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -6885,6 +6975,11 @@
       <c r="H14" s="3" t="n">
         <v>1250</v>
       </c>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -6913,6 +7008,11 @@
       <c r="H15" s="3" t="n">
         <v>1250</v>
       </c>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -6941,6 +7041,11 @@
       <c r="H16" s="3" t="n">
         <v>2000</v>
       </c>
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -6969,6 +7074,11 @@
       <c r="H17" s="3" t="n">
         <v>2000</v>
       </c>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -6997,6 +7107,11 @@
       <c r="H18" s="3" t="n">
         <v>2000</v>
       </c>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr"/>
+      <c r="L18" s="3" t="inlineStr"/>
+      <c r="M18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -7025,6 +7140,11 @@
       <c r="H19" s="3" t="n">
         <v>3250</v>
       </c>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -7053,6 +7173,11 @@
       <c r="H20" s="3" t="n">
         <v>5000</v>
       </c>
+      <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -7081,6 +7206,11 @@
       <c r="H21" s="3" t="n">
         <v>5000</v>
       </c>
+      <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr"/>
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -7109,6 +7239,11 @@
       <c r="H22" s="3" t="n">
         <v>8000</v>
       </c>
+      <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -7137,6 +7272,11 @@
       <c r="H23" s="3" t="n">
         <v>8000</v>
       </c>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr"/>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -7165,6 +7305,11 @@
       <c r="H24" s="3" t="n">
         <v>12500</v>
       </c>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
+      <c r="K24" s="3" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr"/>
+      <c r="M24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -7193,6 +7338,11 @@
       <c r="H25" s="3" t="n">
         <v>12500</v>
       </c>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -7221,6 +7371,11 @@
       <c r="H26" s="3" t="n">
         <v>12500</v>
       </c>
+      <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -7249,6 +7404,11 @@
       <c r="H27" s="3" t="n">
         <v>20000</v>
       </c>
+      <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -7277,6 +7437,11 @@
       <c r="H28" s="3" t="n">
         <v>32500</v>
       </c>
+      <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr"/>
+      <c r="M28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -7305,6 +7470,11 @@
       <c r="H29" s="3" t="n">
         <v>32500</v>
       </c>
+      <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr"/>
+      <c r="K29" s="3" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr"/>
+      <c r="M29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -7333,6 +7503,11 @@
       <c r="H30" s="3" t="n">
         <v>50000</v>
       </c>
+      <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr"/>
+      <c r="M30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -7361,6 +7536,11 @@
       <c r="H31" s="3" t="n">
         <v>50000</v>
       </c>
+      <c r="I31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr"/>
+      <c r="K31" s="3" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr"/>
+      <c r="M31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -7389,6 +7569,11 @@
       <c r="H32" s="3" t="n">
         <v>400</v>
       </c>
+      <c r="I32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="inlineStr"/>
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -7417,6 +7602,11 @@
       <c r="H33" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="I33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr"/>
+      <c r="M33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -7445,6 +7635,11 @@
       <c r="H34" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr"/>
+      <c r="M34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -7473,6 +7668,11 @@
       <c r="H35" s="3" t="n">
         <v>750</v>
       </c>
+      <c r="I35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr"/>
+      <c r="K35" s="3" t="inlineStr"/>
+      <c r="L35" s="3" t="inlineStr"/>
+      <c r="M35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -7501,6 +7701,11 @@
       <c r="H36" s="3" t="n">
         <v>1250</v>
       </c>
+      <c r="I36" s="3" t="inlineStr"/>
+      <c r="J36" s="3" t="inlineStr"/>
+      <c r="K36" s="3" t="inlineStr"/>
+      <c r="L36" s="3" t="inlineStr"/>
+      <c r="M36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -7529,6 +7734,11 @@
       <c r="H37" s="3" t="n">
         <v>2000</v>
       </c>
+      <c r="I37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr"/>
+      <c r="K37" s="3" t="inlineStr"/>
+      <c r="L37" s="3" t="inlineStr"/>
+      <c r="M37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -7557,6 +7767,11 @@
       <c r="H38" s="3" t="n">
         <v>3250</v>
       </c>
+      <c r="I38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr"/>
+      <c r="M38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -7585,6 +7800,11 @@
       <c r="H39" s="3" t="n">
         <v>5000</v>
       </c>
+      <c r="I39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -7613,6 +7833,11 @@
       <c r="H40" s="3" t="n">
         <v>8000</v>
       </c>
+      <c r="I40" s="3" t="inlineStr"/>
+      <c r="J40" s="3" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr"/>
+      <c r="L40" s="3" t="inlineStr"/>
+      <c r="M40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -7641,6 +7866,11 @@
       <c r="H41" s="3" t="n">
         <v>12500</v>
       </c>
+      <c r="I41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr"/>
+      <c r="K41" s="3" t="inlineStr"/>
+      <c r="L41" s="3" t="inlineStr"/>
+      <c r="M41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -7669,6 +7899,11 @@
       <c r="H42" s="3" t="n">
         <v>20000</v>
       </c>
+      <c r="I42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr"/>
+      <c r="K42" s="3" t="inlineStr"/>
+      <c r="L42" s="3" t="inlineStr"/>
+      <c r="M42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -7697,6 +7932,11 @@
       <c r="H43" s="3" t="n">
         <v>32500</v>
       </c>
+      <c r="I43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="inlineStr"/>
+      <c r="K43" s="3" t="inlineStr"/>
+      <c r="L43" s="3" t="inlineStr"/>
+      <c r="M43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -7725,6 +7965,11 @@
       <c r="H44" s="3" t="n">
         <v>50000</v>
       </c>
+      <c r="I44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr"/>
+      <c r="K44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr"/>
+      <c r="M44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -7753,6 +7998,11 @@
       <c r="H45" s="3" t="n">
         <v>80000</v>
       </c>
+      <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr"/>
+      <c r="K45" s="3" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr"/>
+      <c r="M45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -7781,6 +8031,11 @@
       <c r="H46" s="3" t="n">
         <v>125000</v>
       </c>
+      <c r="I46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="inlineStr"/>
+      <c r="K46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr"/>
+      <c r="M46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -7809,6 +8064,11 @@
       <c r="H47" s="3" t="n">
         <v>50000</v>
       </c>
+      <c r="I47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr"/>
+      <c r="K47" s="3" t="inlineStr"/>
+      <c r="L47" s="3" t="inlineStr"/>
+      <c r="M47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -7837,6 +8097,11 @@
       <c r="H48" s="3" t="n">
         <v>125000</v>
       </c>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr"/>
+      <c r="K48" s="3" t="inlineStr"/>
+      <c r="L48" s="3" t="inlineStr"/>
+      <c r="M48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -7865,6 +8130,11 @@
       <c r="H49" s="3" t="n">
         <v>80000</v>
       </c>
+      <c r="I49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr"/>
+      <c r="K49" s="3" t="inlineStr"/>
+      <c r="L49" s="3" t="inlineStr"/>
+      <c r="M49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -7893,6 +8163,11 @@
       <c r="H50" s="3" t="n">
         <v>20000</v>
       </c>
+      <c r="I50" s="3" t="inlineStr"/>
+      <c r="J50" s="3" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr"/>
+      <c r="L50" s="3" t="inlineStr"/>
+      <c r="M50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -7921,6 +8196,11 @@
       <c r="H51" s="3" t="n">
         <v>125000</v>
       </c>
+      <c r="I51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr"/>
+      <c r="K51" s="3" t="inlineStr"/>
+      <c r="L51" s="3" t="inlineStr"/>
+      <c r="M51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -7949,6 +8229,11 @@
       <c r="H52" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="I52" s="3" t="inlineStr"/>
+      <c r="J52" s="3" t="inlineStr"/>
+      <c r="K52" s="3" t="inlineStr"/>
+      <c r="L52" s="3" t="inlineStr"/>
+      <c r="M52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -7977,6 +8262,11 @@
       <c r="H53" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="I53" s="3" t="inlineStr"/>
+      <c r="J53" s="3" t="inlineStr"/>
+      <c r="K53" s="3" t="inlineStr"/>
+      <c r="L53" s="3" t="inlineStr"/>
+      <c r="M53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -8005,6 +8295,11 @@
       <c r="H54" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="I54" s="3" t="inlineStr"/>
+      <c r="J54" s="3" t="inlineStr"/>
+      <c r="K54" s="3" t="inlineStr"/>
+      <c r="L54" s="3" t="inlineStr"/>
+      <c r="M54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -8033,6 +8328,11 @@
       <c r="H55" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I55" s="3" t="inlineStr"/>
+      <c r="J55" s="3" t="inlineStr"/>
+      <c r="K55" s="3" t="inlineStr"/>
+      <c r="L55" s="3" t="inlineStr"/>
+      <c r="M55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -8061,6 +8361,11 @@
       <c r="H56" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I56" s="3" t="inlineStr"/>
+      <c r="J56" s="3" t="inlineStr"/>
+      <c r="K56" s="3" t="inlineStr"/>
+      <c r="L56" s="3" t="inlineStr"/>
+      <c r="M56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -8089,6 +8394,11 @@
       <c r="H57" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I57" s="3" t="inlineStr"/>
+      <c r="J57" s="3" t="inlineStr"/>
+      <c r="K57" s="3" t="inlineStr"/>
+      <c r="L57" s="3" t="inlineStr"/>
+      <c r="M57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -8117,6 +8427,11 @@
       <c r="H58" s="3" t="n">
         <v>400</v>
       </c>
+      <c r="I58" s="3" t="inlineStr"/>
+      <c r="J58" s="3" t="inlineStr"/>
+      <c r="K58" s="3" t="inlineStr"/>
+      <c r="L58" s="3" t="inlineStr"/>
+      <c r="M58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -8145,6 +8460,11 @@
       <c r="H59" s="3" t="n">
         <v>400</v>
       </c>
+      <c r="I59" s="3" t="inlineStr"/>
+      <c r="J59" s="3" t="inlineStr"/>
+      <c r="K59" s="3" t="inlineStr"/>
+      <c r="L59" s="3" t="inlineStr"/>
+      <c r="M59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -8173,6 +8493,11 @@
       <c r="H60" s="3" t="n">
         <v>800</v>
       </c>
+      <c r="I60" s="3" t="inlineStr"/>
+      <c r="J60" s="3" t="inlineStr"/>
+      <c r="K60" s="3" t="inlineStr"/>
+      <c r="L60" s="3" t="inlineStr"/>
+      <c r="M60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -8201,6 +8526,11 @@
       <c r="H61" s="3" t="n">
         <v>800</v>
       </c>
+      <c r="I61" s="3" t="inlineStr"/>
+      <c r="J61" s="3" t="inlineStr"/>
+      <c r="K61" s="3" t="inlineStr"/>
+      <c r="L61" s="3" t="inlineStr"/>
+      <c r="M61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -8229,6 +8559,11 @@
       <c r="H62" s="3" t="n">
         <v>1500</v>
       </c>
+      <c r="I62" s="3" t="inlineStr"/>
+      <c r="J62" s="3" t="inlineStr"/>
+      <c r="K62" s="3" t="inlineStr"/>
+      <c r="L62" s="3" t="inlineStr"/>
+      <c r="M62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -8257,6 +8592,11 @@
       <c r="H63" s="3" t="n">
         <v>1500</v>
       </c>
+      <c r="I63" s="3" t="inlineStr"/>
+      <c r="J63" s="3" t="inlineStr"/>
+      <c r="K63" s="3" t="inlineStr"/>
+      <c r="L63" s="3" t="inlineStr"/>
+      <c r="M63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -8285,6 +8625,11 @@
       <c r="H64" s="3" t="n">
         <v>2500</v>
       </c>
+      <c r="I64" s="3" t="inlineStr"/>
+      <c r="J64" s="3" t="inlineStr"/>
+      <c r="K64" s="3" t="inlineStr"/>
+      <c r="L64" s="3" t="inlineStr"/>
+      <c r="M64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -8313,6 +8658,11 @@
       <c r="H65" s="3" t="n">
         <v>2500</v>
       </c>
+      <c r="I65" s="3" t="inlineStr"/>
+      <c r="J65" s="3" t="inlineStr"/>
+      <c r="K65" s="3" t="inlineStr"/>
+      <c r="L65" s="3" t="inlineStr"/>
+      <c r="M65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -8341,6 +8691,11 @@
       <c r="H66" s="3" t="n">
         <v>4000</v>
       </c>
+      <c r="I66" s="3" t="inlineStr"/>
+      <c r="J66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr"/>
+      <c r="L66" s="3" t="inlineStr"/>
+      <c r="M66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -8369,6 +8724,11 @@
       <c r="H67" s="3" t="n">
         <v>4000</v>
       </c>
+      <c r="I67" s="3" t="inlineStr"/>
+      <c r="J67" s="3" t="inlineStr"/>
+      <c r="K67" s="3" t="inlineStr"/>
+      <c r="L67" s="3" t="inlineStr"/>
+      <c r="M67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -8397,6 +8757,11 @@
       <c r="H68" s="3" t="n">
         <v>4000</v>
       </c>
+      <c r="I68" s="3" t="inlineStr"/>
+      <c r="J68" s="3" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr"/>
+      <c r="L68" s="3" t="inlineStr"/>
+      <c r="M68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -8425,6 +8790,11 @@
       <c r="H69" s="3" t="n">
         <v>6500</v>
       </c>
+      <c r="I69" s="3" t="inlineStr"/>
+      <c r="J69" s="3" t="inlineStr"/>
+      <c r="K69" s="3" t="inlineStr"/>
+      <c r="L69" s="3" t="inlineStr"/>
+      <c r="M69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -8453,6 +8823,11 @@
       <c r="H70" s="3" t="n">
         <v>10000</v>
       </c>
+      <c r="I70" s="3" t="inlineStr"/>
+      <c r="J70" s="3" t="inlineStr"/>
+      <c r="K70" s="3" t="inlineStr"/>
+      <c r="L70" s="3" t="inlineStr"/>
+      <c r="M70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -8481,6 +8856,11 @@
       <c r="H71" s="3" t="n">
         <v>10000</v>
       </c>
+      <c r="I71" s="3" t="inlineStr"/>
+      <c r="J71" s="3" t="inlineStr"/>
+      <c r="K71" s="3" t="inlineStr"/>
+      <c r="L71" s="3" t="inlineStr"/>
+      <c r="M71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -8509,6 +8889,11 @@
       <c r="H72" s="3" t="n">
         <v>16000</v>
       </c>
+      <c r="I72" s="3" t="inlineStr"/>
+      <c r="J72" s="3" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr"/>
+      <c r="L72" s="3" t="inlineStr"/>
+      <c r="M72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -8537,6 +8922,11 @@
       <c r="H73" s="3" t="n">
         <v>16000</v>
       </c>
+      <c r="I73" s="3" t="inlineStr"/>
+      <c r="J73" s="3" t="inlineStr"/>
+      <c r="K73" s="3" t="inlineStr"/>
+      <c r="L73" s="3" t="inlineStr"/>
+      <c r="M73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -8565,6 +8955,11 @@
       <c r="H74" s="3" t="n">
         <v>25000</v>
       </c>
+      <c r="I74" s="3" t="inlineStr"/>
+      <c r="J74" s="3" t="inlineStr"/>
+      <c r="K74" s="3" t="inlineStr"/>
+      <c r="L74" s="3" t="inlineStr"/>
+      <c r="M74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -8593,6 +8988,11 @@
       <c r="H75" s="3" t="n">
         <v>25000</v>
       </c>
+      <c r="I75" s="3" t="inlineStr"/>
+      <c r="J75" s="3" t="inlineStr"/>
+      <c r="K75" s="3" t="inlineStr"/>
+      <c r="L75" s="3" t="inlineStr"/>
+      <c r="M75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -8621,6 +9021,11 @@
       <c r="H76" s="3" t="n">
         <v>25000</v>
       </c>
+      <c r="I76" s="3" t="inlineStr"/>
+      <c r="J76" s="3" t="inlineStr"/>
+      <c r="K76" s="3" t="inlineStr"/>
+      <c r="L76" s="3" t="inlineStr"/>
+      <c r="M76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -8649,6 +9054,11 @@
       <c r="H77" s="3" t="n">
         <v>40000</v>
       </c>
+      <c r="I77" s="3" t="inlineStr"/>
+      <c r="J77" s="3" t="inlineStr"/>
+      <c r="K77" s="3" t="inlineStr"/>
+      <c r="L77" s="3" t="inlineStr"/>
+      <c r="M77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -8677,6 +9087,11 @@
       <c r="H78" s="3" t="n">
         <v>65000</v>
       </c>
+      <c r="I78" s="3" t="inlineStr"/>
+      <c r="J78" s="3" t="inlineStr"/>
+      <c r="K78" s="3" t="inlineStr"/>
+      <c r="L78" s="3" t="inlineStr"/>
+      <c r="M78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -8705,6 +9120,11 @@
       <c r="H79" s="3" t="n">
         <v>65000</v>
       </c>
+      <c r="I79" s="3" t="inlineStr"/>
+      <c r="J79" s="3" t="inlineStr"/>
+      <c r="K79" s="3" t="inlineStr"/>
+      <c r="L79" s="3" t="inlineStr"/>
+      <c r="M79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -8733,6 +9153,11 @@
       <c r="H80" s="3" t="n">
         <v>100000</v>
       </c>
+      <c r="I80" s="3" t="inlineStr"/>
+      <c r="J80" s="3" t="inlineStr"/>
+      <c r="K80" s="3" t="inlineStr"/>
+      <c r="L80" s="3" t="inlineStr"/>
+      <c r="M80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -8761,6 +9186,11 @@
       <c r="H81" s="3" t="n">
         <v>100000</v>
       </c>
+      <c r="I81" s="3" t="inlineStr"/>
+      <c r="J81" s="3" t="inlineStr"/>
+      <c r="K81" s="3" t="inlineStr"/>
+      <c r="L81" s="3" t="inlineStr"/>
+      <c r="M81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -8789,6 +9219,11 @@
       <c r="H82" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I82" s="3" t="inlineStr"/>
+      <c r="J82" s="3" t="inlineStr"/>
+      <c r="K82" s="3" t="inlineStr"/>
+      <c r="L82" s="3" t="inlineStr"/>
+      <c r="M82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -8817,6 +9252,11 @@
       <c r="H83" s="3" t="n">
         <v>400</v>
       </c>
+      <c r="I83" s="3" t="inlineStr"/>
+      <c r="J83" s="3" t="inlineStr"/>
+      <c r="K83" s="3" t="inlineStr"/>
+      <c r="L83" s="3" t="inlineStr"/>
+      <c r="M83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -8845,6 +9285,11 @@
       <c r="H84" s="3" t="n">
         <v>1500</v>
       </c>
+      <c r="I84" s="3" t="inlineStr"/>
+      <c r="J84" s="3" t="inlineStr"/>
+      <c r="K84" s="3" t="inlineStr"/>
+      <c r="L84" s="3" t="inlineStr"/>
+      <c r="M84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -8873,6 +9318,11 @@
       <c r="H85" s="3" t="n">
         <v>2500</v>
       </c>
+      <c r="I85" s="3" t="inlineStr"/>
+      <c r="J85" s="3" t="inlineStr"/>
+      <c r="K85" s="3" t="inlineStr"/>
+      <c r="L85" s="3" t="inlineStr"/>
+      <c r="M85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -8901,6 +9351,11 @@
       <c r="H86" s="3" t="n">
         <v>4000</v>
       </c>
+      <c r="I86" s="3" t="inlineStr"/>
+      <c r="J86" s="3" t="inlineStr"/>
+      <c r="K86" s="3" t="inlineStr"/>
+      <c r="L86" s="3" t="inlineStr"/>
+      <c r="M86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -8929,6 +9384,11 @@
       <c r="H87" s="3" t="n">
         <v>6500</v>
       </c>
+      <c r="I87" s="3" t="inlineStr"/>
+      <c r="J87" s="3" t="inlineStr"/>
+      <c r="K87" s="3" t="inlineStr"/>
+      <c r="L87" s="3" t="inlineStr"/>
+      <c r="M87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -8957,6 +9417,11 @@
       <c r="H88" s="3" t="n">
         <v>10000</v>
       </c>
+      <c r="I88" s="3" t="inlineStr"/>
+      <c r="J88" s="3" t="inlineStr"/>
+      <c r="K88" s="3" t="inlineStr"/>
+      <c r="L88" s="3" t="inlineStr"/>
+      <c r="M88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -8985,6 +9450,11 @@
       <c r="H89" s="3" t="n">
         <v>16000</v>
       </c>
+      <c r="I89" s="3" t="inlineStr"/>
+      <c r="J89" s="3" t="inlineStr"/>
+      <c r="K89" s="3" t="inlineStr"/>
+      <c r="L89" s="3" t="inlineStr"/>
+      <c r="M89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -9013,6 +9483,11 @@
       <c r="H90" s="3" t="n">
         <v>25000</v>
       </c>
+      <c r="I90" s="3" t="inlineStr"/>
+      <c r="J90" s="3" t="inlineStr"/>
+      <c r="K90" s="3" t="inlineStr"/>
+      <c r="L90" s="3" t="inlineStr"/>
+      <c r="M90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -9041,6 +9516,11 @@
       <c r="H91" s="3" t="n">
         <v>40000</v>
       </c>
+      <c r="I91" s="3" t="inlineStr"/>
+      <c r="J91" s="3" t="inlineStr"/>
+      <c r="K91" s="3" t="inlineStr"/>
+      <c r="L91" s="3" t="inlineStr"/>
+      <c r="M91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -9069,6 +9549,11 @@
       <c r="H92" s="3" t="n">
         <v>65000</v>
       </c>
+      <c r="I92" s="3" t="inlineStr"/>
+      <c r="J92" s="3" t="inlineStr"/>
+      <c r="K92" s="3" t="inlineStr"/>
+      <c r="L92" s="3" t="inlineStr"/>
+      <c r="M92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -9097,6 +9582,11 @@
       <c r="H93" s="3" t="n">
         <v>100000</v>
       </c>
+      <c r="I93" s="3" t="inlineStr"/>
+      <c r="J93" s="3" t="inlineStr"/>
+      <c r="K93" s="3" t="inlineStr"/>
+      <c r="L93" s="3" t="inlineStr"/>
+      <c r="M93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -9125,6 +9615,11 @@
       <c r="H94" s="3" t="n">
         <v>160000</v>
       </c>
+      <c r="I94" s="3" t="inlineStr"/>
+      <c r="J94" s="3" t="inlineStr"/>
+      <c r="K94" s="3" t="inlineStr"/>
+      <c r="L94" s="3" t="inlineStr"/>
+      <c r="M94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -9153,6 +9648,11 @@
       <c r="H95" s="3" t="n">
         <v>250000</v>
       </c>
+      <c r="I95" s="3" t="inlineStr"/>
+      <c r="J95" s="3" t="inlineStr"/>
+      <c r="K95" s="3" t="inlineStr"/>
+      <c r="L95" s="3" t="inlineStr"/>
+      <c r="M95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -9181,6 +9681,11 @@
       <c r="H96" s="3" t="n">
         <v>40000</v>
       </c>
+      <c r="I96" s="3" t="inlineStr"/>
+      <c r="J96" s="3" t="inlineStr"/>
+      <c r="K96" s="3" t="inlineStr"/>
+      <c r="L96" s="3" t="inlineStr"/>
+      <c r="M96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -9209,6 +9714,11 @@
       <c r="H97" s="3" t="n">
         <v>250000</v>
       </c>
+      <c r="I97" s="3" t="inlineStr"/>
+      <c r="J97" s="3" t="inlineStr"/>
+      <c r="K97" s="3" t="inlineStr"/>
+      <c r="L97" s="3" t="inlineStr"/>
+      <c r="M97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -9237,6 +9747,11 @@
       <c r="H98" s="3" t="n">
         <v>25000</v>
       </c>
+      <c r="I98" s="3" t="inlineStr"/>
+      <c r="J98" s="3" t="inlineStr"/>
+      <c r="K98" s="3" t="inlineStr"/>
+      <c r="L98" s="3" t="inlineStr"/>
+      <c r="M98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -9265,6 +9780,11 @@
       <c r="H99" s="3" t="n">
         <v>100000</v>
       </c>
+      <c r="I99" s="3" t="inlineStr"/>
+      <c r="J99" s="3" t="inlineStr"/>
+      <c r="K99" s="3" t="inlineStr"/>
+      <c r="L99" s="3" t="inlineStr"/>
+      <c r="M99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -9293,6 +9813,11 @@
       <c r="H100" s="3" t="n">
         <v>160000</v>
       </c>
+      <c r="I100" s="3" t="inlineStr"/>
+      <c r="J100" s="3" t="inlineStr"/>
+      <c r="K100" s="3" t="inlineStr"/>
+      <c r="L100" s="3" t="inlineStr"/>
+      <c r="M100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -9321,6 +9846,11 @@
       <c r="H101" s="3" t="n">
         <v>250000</v>
       </c>
+      <c r="I101" s="3" t="inlineStr"/>
+      <c r="J101" s="3" t="inlineStr"/>
+      <c r="K101" s="3" t="inlineStr"/>
+      <c r="L101" s="3" t="inlineStr"/>
+      <c r="M101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -9345,6 +9875,11 @@
       </c>
       <c r="G102" s="3" t="inlineStr"/>
       <c r="H102" s="3" t="inlineStr"/>
+      <c r="I102" s="3" t="inlineStr"/>
+      <c r="J102" s="3" t="inlineStr"/>
+      <c r="K102" s="3" t="inlineStr"/>
+      <c r="L102" s="3" t="inlineStr"/>
+      <c r="M102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -9369,6 +9904,11 @@
       </c>
       <c r="G103" s="3" t="inlineStr"/>
       <c r="H103" s="3" t="inlineStr"/>
+      <c r="I103" s="3" t="inlineStr"/>
+      <c r="J103" s="3" t="inlineStr"/>
+      <c r="K103" s="3" t="inlineStr"/>
+      <c r="L103" s="3" t="inlineStr"/>
+      <c r="M103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -9393,6 +9933,11 @@
       </c>
       <c r="G104" s="3" t="inlineStr"/>
       <c r="H104" s="3" t="inlineStr"/>
+      <c r="I104" s="3" t="inlineStr"/>
+      <c r="J104" s="3" t="inlineStr"/>
+      <c r="K104" s="3" t="inlineStr"/>
+      <c r="L104" s="3" t="inlineStr"/>
+      <c r="M104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -9417,6 +9962,11 @@
       </c>
       <c r="G105" s="3" t="inlineStr"/>
       <c r="H105" s="3" t="inlineStr"/>
+      <c r="I105" s="3" t="inlineStr"/>
+      <c r="J105" s="3" t="inlineStr"/>
+      <c r="K105" s="3" t="inlineStr"/>
+      <c r="L105" s="3" t="inlineStr"/>
+      <c r="M105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -9441,6 +9991,11 @@
       </c>
       <c r="G106" s="3" t="inlineStr"/>
       <c r="H106" s="3" t="inlineStr"/>
+      <c r="I106" s="3" t="inlineStr"/>
+      <c r="J106" s="3" t="inlineStr"/>
+      <c r="K106" s="3" t="inlineStr"/>
+      <c r="L106" s="3" t="inlineStr"/>
+      <c r="M106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -9465,6 +10020,11 @@
       </c>
       <c r="G107" s="3" t="inlineStr"/>
       <c r="H107" s="3" t="inlineStr"/>
+      <c r="I107" s="3" t="inlineStr"/>
+      <c r="J107" s="3" t="inlineStr"/>
+      <c r="K107" s="3" t="inlineStr"/>
+      <c r="L107" s="3" t="inlineStr"/>
+      <c r="M107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -9489,6 +10049,11 @@
       </c>
       <c r="G108" s="3" t="inlineStr"/>
       <c r="H108" s="3" t="inlineStr"/>
+      <c r="I108" s="3" t="inlineStr"/>
+      <c r="J108" s="3" t="inlineStr"/>
+      <c r="K108" s="3" t="inlineStr"/>
+      <c r="L108" s="3" t="inlineStr"/>
+      <c r="M108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -9513,6 +10078,11 @@
       </c>
       <c r="G109" s="3" t="inlineStr"/>
       <c r="H109" s="3" t="inlineStr"/>
+      <c r="I109" s="3" t="inlineStr"/>
+      <c r="J109" s="3" t="inlineStr"/>
+      <c r="K109" s="3" t="inlineStr"/>
+      <c r="L109" s="3" t="inlineStr"/>
+      <c r="M109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -9537,6 +10107,11 @@
       </c>
       <c r="G110" s="3" t="inlineStr"/>
       <c r="H110" s="3" t="inlineStr"/>
+      <c r="I110" s="3" t="inlineStr"/>
+      <c r="J110" s="3" t="inlineStr"/>
+      <c r="K110" s="3" t="inlineStr"/>
+      <c r="L110" s="3" t="inlineStr"/>
+      <c r="M110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
@@ -9561,6 +10136,11 @@
       </c>
       <c r="G111" s="3" t="inlineStr"/>
       <c r="H111" s="3" t="inlineStr"/>
+      <c r="I111" s="3" t="inlineStr"/>
+      <c r="J111" s="3" t="inlineStr"/>
+      <c r="K111" s="3" t="inlineStr"/>
+      <c r="L111" s="3" t="inlineStr"/>
+      <c r="M111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -9585,6 +10165,11 @@
       </c>
       <c r="G112" s="3" t="inlineStr"/>
       <c r="H112" s="3" t="inlineStr"/>
+      <c r="I112" s="3" t="inlineStr"/>
+      <c r="J112" s="3" t="inlineStr"/>
+      <c r="K112" s="3" t="inlineStr"/>
+      <c r="L112" s="3" t="inlineStr"/>
+      <c r="M112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -9609,6 +10194,11 @@
       </c>
       <c r="G113" s="3" t="inlineStr"/>
       <c r="H113" s="3" t="inlineStr"/>
+      <c r="I113" s="3" t="inlineStr"/>
+      <c r="J113" s="3" t="inlineStr"/>
+      <c r="K113" s="3" t="inlineStr"/>
+      <c r="L113" s="3" t="inlineStr"/>
+      <c r="M113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -9633,6 +10223,11 @@
       </c>
       <c r="G114" s="3" t="inlineStr"/>
       <c r="H114" s="3" t="inlineStr"/>
+      <c r="I114" s="3" t="inlineStr"/>
+      <c r="J114" s="3" t="inlineStr"/>
+      <c r="K114" s="3" t="inlineStr"/>
+      <c r="L114" s="3" t="inlineStr"/>
+      <c r="M114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -9657,6 +10252,11 @@
       </c>
       <c r="G115" s="3" t="inlineStr"/>
       <c r="H115" s="3" t="inlineStr"/>
+      <c r="I115" s="3" t="inlineStr"/>
+      <c r="J115" s="3" t="inlineStr"/>
+      <c r="K115" s="3" t="inlineStr"/>
+      <c r="L115" s="3" t="inlineStr"/>
+      <c r="M115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -9681,6 +10281,11 @@
       </c>
       <c r="G116" s="3" t="inlineStr"/>
       <c r="H116" s="3" t="inlineStr"/>
+      <c r="I116" s="3" t="inlineStr"/>
+      <c r="J116" s="3" t="inlineStr"/>
+      <c r="K116" s="3" t="inlineStr"/>
+      <c r="L116" s="3" t="inlineStr"/>
+      <c r="M116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -9705,6 +10310,11 @@
       </c>
       <c r="G117" s="3" t="inlineStr"/>
       <c r="H117" s="3" t="inlineStr"/>
+      <c r="I117" s="3" t="inlineStr"/>
+      <c r="J117" s="3" t="inlineStr"/>
+      <c r="K117" s="3" t="inlineStr"/>
+      <c r="L117" s="3" t="inlineStr"/>
+      <c r="M117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -9729,6 +10339,11 @@
       </c>
       <c r="G118" s="3" t="inlineStr"/>
       <c r="H118" s="3" t="inlineStr"/>
+      <c r="I118" s="3" t="inlineStr"/>
+      <c r="J118" s="3" t="inlineStr"/>
+      <c r="K118" s="3" t="inlineStr"/>
+      <c r="L118" s="3" t="inlineStr"/>
+      <c r="M118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -9753,6 +10368,11 @@
       </c>
       <c r="G119" s="3" t="inlineStr"/>
       <c r="H119" s="3" t="inlineStr"/>
+      <c r="I119" s="3" t="inlineStr"/>
+      <c r="J119" s="3" t="inlineStr"/>
+      <c r="K119" s="3" t="inlineStr"/>
+      <c r="L119" s="3" t="inlineStr"/>
+      <c r="M119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -9777,6 +10397,11 @@
       </c>
       <c r="G120" s="3" t="inlineStr"/>
       <c r="H120" s="3" t="inlineStr"/>
+      <c r="I120" s="3" t="inlineStr"/>
+      <c r="J120" s="3" t="inlineStr"/>
+      <c r="K120" s="3" t="inlineStr"/>
+      <c r="L120" s="3" t="inlineStr"/>
+      <c r="M120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -9801,6 +10426,11 @@
       </c>
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="3" t="inlineStr"/>
+      <c r="I121" s="3" t="inlineStr"/>
+      <c r="J121" s="3" t="inlineStr"/>
+      <c r="K121" s="3" t="inlineStr"/>
+      <c r="L121" s="3" t="inlineStr"/>
+      <c r="M121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -9825,6 +10455,11 @@
       </c>
       <c r="G122" s="3" t="inlineStr"/>
       <c r="H122" s="3" t="inlineStr"/>
+      <c r="I122" s="3" t="inlineStr"/>
+      <c r="J122" s="3" t="inlineStr"/>
+      <c r="K122" s="3" t="inlineStr"/>
+      <c r="L122" s="3" t="inlineStr"/>
+      <c r="M122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -9849,6 +10484,11 @@
       </c>
       <c r="G123" s="3" t="inlineStr"/>
       <c r="H123" s="3" t="inlineStr"/>
+      <c r="I123" s="3" t="inlineStr"/>
+      <c r="J123" s="3" t="inlineStr"/>
+      <c r="K123" s="3" t="inlineStr"/>
+      <c r="L123" s="3" t="inlineStr"/>
+      <c r="M123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -9873,6 +10513,11 @@
       </c>
       <c r="G124" s="3" t="inlineStr"/>
       <c r="H124" s="3" t="inlineStr"/>
+      <c r="I124" s="3" t="inlineStr"/>
+      <c r="J124" s="3" t="inlineStr"/>
+      <c r="K124" s="3" t="inlineStr"/>
+      <c r="L124" s="3" t="inlineStr"/>
+      <c r="M124" s="3" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -9897,6 +10542,11 @@
       </c>
       <c r="G125" s="3" t="inlineStr"/>
       <c r="H125" s="3" t="inlineStr"/>
+      <c r="I125" s="3" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr"/>
+      <c r="K125" s="3" t="inlineStr"/>
+      <c r="L125" s="3" t="inlineStr"/>
+      <c r="M125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -9921,6 +10571,11 @@
       </c>
       <c r="G126" s="3" t="inlineStr"/>
       <c r="H126" s="3" t="inlineStr"/>
+      <c r="I126" s="3" t="inlineStr"/>
+      <c r="J126" s="3" t="inlineStr"/>
+      <c r="K126" s="3" t="inlineStr"/>
+      <c r="L126" s="3" t="inlineStr"/>
+      <c r="M126" s="3" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -9945,6 +10600,11 @@
       </c>
       <c r="G127" s="3" t="inlineStr"/>
       <c r="H127" s="3" t="inlineStr"/>
+      <c r="I127" s="3" t="inlineStr"/>
+      <c r="J127" s="3" t="inlineStr"/>
+      <c r="K127" s="3" t="inlineStr"/>
+      <c r="L127" s="3" t="inlineStr"/>
+      <c r="M127" s="3" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -9969,6 +10629,11 @@
       </c>
       <c r="G128" s="3" t="inlineStr"/>
       <c r="H128" s="3" t="inlineStr"/>
+      <c r="I128" s="3" t="inlineStr"/>
+      <c r="J128" s="3" t="inlineStr"/>
+      <c r="K128" s="3" t="inlineStr"/>
+      <c r="L128" s="3" t="inlineStr"/>
+      <c r="M128" s="3" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -9993,6 +10658,11 @@
       </c>
       <c r="G129" s="3" t="inlineStr"/>
       <c r="H129" s="3" t="inlineStr"/>
+      <c r="I129" s="3" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr"/>
+      <c r="K129" s="3" t="inlineStr"/>
+      <c r="L129" s="3" t="inlineStr"/>
+      <c r="M129" s="3" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -10017,6 +10687,11 @@
       </c>
       <c r="G130" s="3" t="inlineStr"/>
       <c r="H130" s="3" t="inlineStr"/>
+      <c r="I130" s="3" t="inlineStr"/>
+      <c r="J130" s="3" t="inlineStr"/>
+      <c r="K130" s="3" t="inlineStr"/>
+      <c r="L130" s="3" t="inlineStr"/>
+      <c r="M130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
@@ -10041,6 +10716,11 @@
       </c>
       <c r="G131" s="3" t="inlineStr"/>
       <c r="H131" s="3" t="inlineStr"/>
+      <c r="I131" s="3" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr"/>
+      <c r="K131" s="3" t="inlineStr"/>
+      <c r="L131" s="3" t="inlineStr"/>
+      <c r="M131" s="3" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
@@ -10065,6 +10745,11 @@
       </c>
       <c r="G132" s="3" t="inlineStr"/>
       <c r="H132" s="3" t="inlineStr"/>
+      <c r="I132" s="3" t="inlineStr"/>
+      <c r="J132" s="3" t="inlineStr"/>
+      <c r="K132" s="3" t="inlineStr"/>
+      <c r="L132" s="3" t="inlineStr"/>
+      <c r="M132" s="3" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
@@ -10089,6 +10774,11 @@
       </c>
       <c r="G133" s="3" t="inlineStr"/>
       <c r="H133" s="3" t="inlineStr"/>
+      <c r="I133" s="3" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr"/>
+      <c r="K133" s="3" t="inlineStr"/>
+      <c r="L133" s="3" t="inlineStr"/>
+      <c r="M133" s="3" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
@@ -10113,6 +10803,11 @@
       </c>
       <c r="G134" s="3" t="inlineStr"/>
       <c r="H134" s="3" t="inlineStr"/>
+      <c r="I134" s="3" t="inlineStr"/>
+      <c r="J134" s="3" t="inlineStr"/>
+      <c r="K134" s="3" t="inlineStr"/>
+      <c r="L134" s="3" t="inlineStr"/>
+      <c r="M134" s="3" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
@@ -10137,6 +10832,11 @@
       </c>
       <c r="G135" s="3" t="inlineStr"/>
       <c r="H135" s="3" t="inlineStr"/>
+      <c r="I135" s="3" t="inlineStr"/>
+      <c r="J135" s="3" t="inlineStr"/>
+      <c r="K135" s="3" t="inlineStr"/>
+      <c r="L135" s="3" t="inlineStr"/>
+      <c r="M135" s="3" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
@@ -10161,6 +10861,11 @@
       </c>
       <c r="G136" s="3" t="inlineStr"/>
       <c r="H136" s="3" t="inlineStr"/>
+      <c r="I136" s="3" t="inlineStr"/>
+      <c r="J136" s="3" t="inlineStr"/>
+      <c r="K136" s="3" t="inlineStr"/>
+      <c r="L136" s="3" t="inlineStr"/>
+      <c r="M136" s="3" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
@@ -10185,6 +10890,11 @@
       </c>
       <c r="G137" s="3" t="inlineStr"/>
       <c r="H137" s="3" t="inlineStr"/>
+      <c r="I137" s="3" t="inlineStr"/>
+      <c r="J137" s="3" t="inlineStr"/>
+      <c r="K137" s="3" t="inlineStr"/>
+      <c r="L137" s="3" t="inlineStr"/>
+      <c r="M137" s="3" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
@@ -10209,6 +10919,11 @@
       </c>
       <c r="G138" s="3" t="inlineStr"/>
       <c r="H138" s="3" t="inlineStr"/>
+      <c r="I138" s="3" t="inlineStr"/>
+      <c r="J138" s="3" t="inlineStr"/>
+      <c r="K138" s="3" t="inlineStr"/>
+      <c r="L138" s="3" t="inlineStr"/>
+      <c r="M138" s="3" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
@@ -10233,6 +10948,11 @@
       </c>
       <c r="G139" s="3" t="inlineStr"/>
       <c r="H139" s="3" t="inlineStr"/>
+      <c r="I139" s="3" t="inlineStr"/>
+      <c r="J139" s="3" t="inlineStr"/>
+      <c r="K139" s="3" t="inlineStr"/>
+      <c r="L139" s="3" t="inlineStr"/>
+      <c r="M139" s="3" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
@@ -10257,6 +10977,11 @@
       </c>
       <c r="G140" s="3" t="inlineStr"/>
       <c r="H140" s="3" t="inlineStr"/>
+      <c r="I140" s="3" t="inlineStr"/>
+      <c r="J140" s="3" t="inlineStr"/>
+      <c r="K140" s="3" t="inlineStr"/>
+      <c r="L140" s="3" t="inlineStr"/>
+      <c r="M140" s="3" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
@@ -10281,6 +11006,11 @@
       </c>
       <c r="G141" s="3" t="inlineStr"/>
       <c r="H141" s="3" t="inlineStr"/>
+      <c r="I141" s="3" t="inlineStr"/>
+      <c r="J141" s="3" t="inlineStr"/>
+      <c r="K141" s="3" t="inlineStr"/>
+      <c r="L141" s="3" t="inlineStr"/>
+      <c r="M141" s="3" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n">
@@ -10305,6 +11035,11 @@
       </c>
       <c r="G142" s="3" t="inlineStr"/>
       <c r="H142" s="3" t="inlineStr"/>
+      <c r="I142" s="3" t="inlineStr"/>
+      <c r="J142" s="3" t="inlineStr"/>
+      <c r="K142" s="3" t="inlineStr"/>
+      <c r="L142" s="3" t="inlineStr"/>
+      <c r="M142" s="3" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
@@ -10329,6 +11064,11 @@
       </c>
       <c r="G143" s="3" t="inlineStr"/>
       <c r="H143" s="3" t="inlineStr"/>
+      <c r="I143" s="3" t="inlineStr"/>
+      <c r="J143" s="3" t="inlineStr"/>
+      <c r="K143" s="3" t="inlineStr"/>
+      <c r="L143" s="3" t="inlineStr"/>
+      <c r="M143" s="3" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
@@ -10353,6 +11093,11 @@
       </c>
       <c r="G144" s="3" t="inlineStr"/>
       <c r="H144" s="3" t="inlineStr"/>
+      <c r="I144" s="3" t="inlineStr"/>
+      <c r="J144" s="3" t="inlineStr"/>
+      <c r="K144" s="3" t="inlineStr"/>
+      <c r="L144" s="3" t="inlineStr"/>
+      <c r="M144" s="3" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
@@ -10377,6 +11122,11 @@
       </c>
       <c r="G145" s="3" t="inlineStr"/>
       <c r="H145" s="3" t="inlineStr"/>
+      <c r="I145" s="3" t="inlineStr"/>
+      <c r="J145" s="3" t="inlineStr"/>
+      <c r="K145" s="3" t="inlineStr"/>
+      <c r="L145" s="3" t="inlineStr"/>
+      <c r="M145" s="3" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
@@ -10401,6 +11151,11 @@
       </c>
       <c r="G146" s="3" t="inlineStr"/>
       <c r="H146" s="3" t="inlineStr"/>
+      <c r="I146" s="3" t="inlineStr"/>
+      <c r="J146" s="3" t="inlineStr"/>
+      <c r="K146" s="3" t="inlineStr"/>
+      <c r="L146" s="3" t="inlineStr"/>
+      <c r="M146" s="3" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n">
@@ -10425,6 +11180,11 @@
       </c>
       <c r="G147" s="3" t="inlineStr"/>
       <c r="H147" s="3" t="inlineStr"/>
+      <c r="I147" s="3" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr"/>
+      <c r="K147" s="3" t="inlineStr"/>
+      <c r="L147" s="3" t="inlineStr"/>
+      <c r="M147" s="3" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
@@ -10449,6 +11209,11 @@
       </c>
       <c r="G148" s="3" t="inlineStr"/>
       <c r="H148" s="3" t="inlineStr"/>
+      <c r="I148" s="3" t="inlineStr"/>
+      <c r="J148" s="3" t="inlineStr"/>
+      <c r="K148" s="3" t="inlineStr"/>
+      <c r="L148" s="3" t="inlineStr"/>
+      <c r="M148" s="3" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n">
@@ -10473,6 +11238,11 @@
       </c>
       <c r="G149" s="3" t="inlineStr"/>
       <c r="H149" s="3" t="inlineStr"/>
+      <c r="I149" s="3" t="inlineStr"/>
+      <c r="J149" s="3" t="inlineStr"/>
+      <c r="K149" s="3" t="inlineStr"/>
+      <c r="L149" s="3" t="inlineStr"/>
+      <c r="M149" s="3" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n">
@@ -10497,6 +11267,11 @@
       </c>
       <c r="G150" s="3" t="inlineStr"/>
       <c r="H150" s="3" t="inlineStr"/>
+      <c r="I150" s="3" t="inlineStr"/>
+      <c r="J150" s="3" t="inlineStr"/>
+      <c r="K150" s="3" t="inlineStr"/>
+      <c r="L150" s="3" t="inlineStr"/>
+      <c r="M150" s="3" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n">
@@ -10521,6 +11296,11 @@
       </c>
       <c r="G151" s="3" t="inlineStr"/>
       <c r="H151" s="3" t="inlineStr"/>
+      <c r="I151" s="3" t="inlineStr"/>
+      <c r="J151" s="3" t="inlineStr"/>
+      <c r="K151" s="3" t="inlineStr"/>
+      <c r="L151" s="3" t="inlineStr"/>
+      <c r="M151" s="3" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n">
@@ -10547,8 +11327,21 @@
         <v>7</v>
       </c>
       <c r="H152" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="I152" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J152" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="K152" s="3" t="inlineStr"/>
+      <c r="L152" s="3" t="inlineStr">
+        <is>
+          <t>15101:100</t>
+        </is>
+      </c>
+      <c r="M152" s="3" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="n">
@@ -10575,8 +11368,21 @@
         <v>7</v>
       </c>
       <c r="H153" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="I153" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J153" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="K153" s="3" t="inlineStr"/>
+      <c r="L153" s="3" t="inlineStr">
+        <is>
+          <t>15101:100</t>
+        </is>
+      </c>
+      <c r="M153" s="3" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n">
@@ -10603,8 +11409,21 @@
         <v>7</v>
       </c>
       <c r="H154" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="I154" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J154" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="K154" s="3" t="inlineStr"/>
+      <c r="L154" s="3" t="inlineStr">
+        <is>
+          <t>15101:100</t>
+        </is>
+      </c>
+      <c r="M154" s="3" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n">
@@ -10631,8 +11450,21 @@
         <v>7</v>
       </c>
       <c r="H155" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="I155" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J155" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="K155" s="3" t="inlineStr"/>
+      <c r="L155" s="3" t="inlineStr">
+        <is>
+          <t>15101:100</t>
+        </is>
+      </c>
+      <c r="M155" s="3" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
@@ -10659,8 +11491,21 @@
         <v>7</v>
       </c>
       <c r="H156" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="I156" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J156" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="K156" s="3" t="inlineStr"/>
+      <c r="L156" s="3" t="inlineStr">
+        <is>
+          <t>15102:100</t>
+        </is>
+      </c>
+      <c r="M156" s="3" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n">
@@ -10687,8 +11532,21 @@
         <v>7</v>
       </c>
       <c r="H157" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I157" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J157" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="K157" s="3" t="inlineStr"/>
+      <c r="L157" s="3" t="inlineStr">
+        <is>
+          <t>15102:100</t>
+        </is>
+      </c>
+      <c r="M157" s="3" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n">
@@ -10715,8 +11573,21 @@
         <v>7</v>
       </c>
       <c r="H158" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="I158" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J158" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="K158" s="3" t="inlineStr"/>
+      <c r="L158" s="3" t="inlineStr">
+        <is>
+          <t>15102:100</t>
+        </is>
+      </c>
+      <c r="M158" s="3" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="n">
@@ -10743,8 +11614,21 @@
         <v>7</v>
       </c>
       <c r="H159" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="I159" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J159" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="K159" s="3" t="inlineStr"/>
+      <c r="L159" s="3" t="inlineStr">
+        <is>
+          <t>15102:100</t>
+        </is>
+      </c>
+      <c r="M159" s="3" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n">
@@ -10771,8 +11655,21 @@
         <v>7</v>
       </c>
       <c r="H160" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="I160" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="J160" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K160" s="3" t="inlineStr"/>
+      <c r="L160" s="3" t="inlineStr">
+        <is>
+          <t>15104:100</t>
+        </is>
+      </c>
+      <c r="M160" s="3" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n">
@@ -10799,8 +11696,21 @@
         <v>7</v>
       </c>
       <c r="H161" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="I161" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="J161" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K161" s="3" t="inlineStr"/>
+      <c r="L161" s="3" t="inlineStr">
+        <is>
+          <t>15104:100</t>
+        </is>
+      </c>
+      <c r="M161" s="3" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n">
@@ -10827,8 +11737,21 @@
         <v>7</v>
       </c>
       <c r="H162" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="I162" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="J162" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K162" s="3" t="inlineStr"/>
+      <c r="L162" s="3" t="inlineStr">
+        <is>
+          <t>15104:100</t>
+        </is>
+      </c>
+      <c r="M162" s="3" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="n">
@@ -10855,8 +11778,21 @@
         <v>7</v>
       </c>
       <c r="H163" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="I163" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="J163" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K163" s="3" t="inlineStr"/>
+      <c r="L163" s="3" t="inlineStr">
+        <is>
+          <t>15104:100</t>
+        </is>
+      </c>
+      <c r="M163" s="3" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n">
@@ -10883,8 +11819,21 @@
         <v>7</v>
       </c>
       <c r="H164" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="I164" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="J164" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="K164" s="3" t="inlineStr"/>
+      <c r="L164" s="3" t="inlineStr">
+        <is>
+          <t>15108:100</t>
+        </is>
+      </c>
+      <c r="M164" s="3" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n">
@@ -10911,8 +11860,21 @@
         <v>7</v>
       </c>
       <c r="H165" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="I165" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="J165" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="K165" s="3" t="inlineStr"/>
+      <c r="L165" s="3" t="inlineStr">
+        <is>
+          <t>15108:100</t>
+        </is>
+      </c>
+      <c r="M165" s="3" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n">
@@ -10939,8 +11901,21 @@
         <v>7</v>
       </c>
       <c r="H166" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="I166" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="J166" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="K166" s="3" t="inlineStr"/>
+      <c r="L166" s="3" t="inlineStr">
+        <is>
+          <t>15108:100</t>
+        </is>
+      </c>
+      <c r="M166" s="3" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n">
@@ -10967,8 +11942,21 @@
         <v>7</v>
       </c>
       <c r="H167" s="3" t="n">
-        <v>15101</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="I167" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="J167" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="K167" s="3" t="inlineStr"/>
+      <c r="L167" s="3" t="inlineStr">
+        <is>
+          <t>15108:100</t>
+        </is>
+      </c>
+      <c r="M167" s="3" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n">
@@ -10993,6 +11981,11 @@
       </c>
       <c r="G168" s="3" t="inlineStr"/>
       <c r="H168" s="3" t="inlineStr"/>
+      <c r="I168" s="3" t="inlineStr"/>
+      <c r="J168" s="3" t="inlineStr"/>
+      <c r="K168" s="3" t="inlineStr"/>
+      <c r="L168" s="3" t="inlineStr"/>
+      <c r="M168" s="3" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n">
@@ -11017,6 +12010,11 @@
       </c>
       <c r="G169" s="3" t="inlineStr"/>
       <c r="H169" s="3" t="inlineStr"/>
+      <c r="I169" s="3" t="inlineStr"/>
+      <c r="J169" s="3" t="inlineStr"/>
+      <c r="K169" s="3" t="inlineStr"/>
+      <c r="L169" s="3" t="inlineStr"/>
+      <c r="M169" s="3" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n">
@@ -11041,6 +12039,11 @@
       </c>
       <c r="G170" s="3" t="inlineStr"/>
       <c r="H170" s="3" t="inlineStr"/>
+      <c r="I170" s="3" t="inlineStr"/>
+      <c r="J170" s="3" t="inlineStr"/>
+      <c r="K170" s="3" t="inlineStr"/>
+      <c r="L170" s="3" t="inlineStr"/>
+      <c r="M170" s="3" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n">
@@ -11065,6 +12068,11 @@
       </c>
       <c r="G171" s="3" t="inlineStr"/>
       <c r="H171" s="3" t="inlineStr"/>
+      <c r="I171" s="3" t="inlineStr"/>
+      <c r="J171" s="3" t="inlineStr"/>
+      <c r="K171" s="3" t="inlineStr"/>
+      <c r="L171" s="3" t="inlineStr"/>
+      <c r="M171" s="3" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n">
@@ -11089,6 +12097,11 @@
       </c>
       <c r="G172" s="3" t="inlineStr"/>
       <c r="H172" s="3" t="inlineStr"/>
+      <c r="I172" s="3" t="inlineStr"/>
+      <c r="J172" s="3" t="inlineStr"/>
+      <c r="K172" s="3" t="inlineStr"/>
+      <c r="L172" s="3" t="inlineStr"/>
+      <c r="M172" s="3" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n">
@@ -11113,6 +12126,11 @@
       </c>
       <c r="G173" s="3" t="inlineStr"/>
       <c r="H173" s="3" t="inlineStr"/>
+      <c r="I173" s="3" t="inlineStr"/>
+      <c r="J173" s="3" t="inlineStr"/>
+      <c r="K173" s="3" t="inlineStr"/>
+      <c r="L173" s="3" t="inlineStr"/>
+      <c r="M173" s="3" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n">
@@ -11137,6 +12155,11 @@
       </c>
       <c r="G174" s="3" t="inlineStr"/>
       <c r="H174" s="3" t="inlineStr"/>
+      <c r="I174" s="3" t="inlineStr"/>
+      <c r="J174" s="3" t="inlineStr"/>
+      <c r="K174" s="3" t="inlineStr"/>
+      <c r="L174" s="3" t="inlineStr"/>
+      <c r="M174" s="3" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n">
@@ -11161,6 +12184,11 @@
       </c>
       <c r="G175" s="3" t="inlineStr"/>
       <c r="H175" s="3" t="inlineStr"/>
+      <c r="I175" s="3" t="inlineStr"/>
+      <c r="J175" s="3" t="inlineStr"/>
+      <c r="K175" s="3" t="inlineStr"/>
+      <c r="L175" s="3" t="inlineStr"/>
+      <c r="M175" s="3" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n">
@@ -11185,6 +12213,11 @@
       </c>
       <c r="G176" s="3" t="inlineStr"/>
       <c r="H176" s="3" t="inlineStr"/>
+      <c r="I176" s="3" t="inlineStr"/>
+      <c r="J176" s="3" t="inlineStr"/>
+      <c r="K176" s="3" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr"/>
+      <c r="M176" s="3" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n">
@@ -11209,6 +12242,11 @@
       </c>
       <c r="G177" s="3" t="inlineStr"/>
       <c r="H177" s="3" t="inlineStr"/>
+      <c r="I177" s="3" t="inlineStr"/>
+      <c r="J177" s="3" t="inlineStr"/>
+      <c r="K177" s="3" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr"/>
+      <c r="M177" s="3" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n">
@@ -11233,6 +12271,11 @@
       </c>
       <c r="G178" s="3" t="inlineStr"/>
       <c r="H178" s="3" t="inlineStr"/>
+      <c r="I178" s="3" t="inlineStr"/>
+      <c r="J178" s="3" t="inlineStr"/>
+      <c r="K178" s="3" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr"/>
+      <c r="M178" s="3" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n">
@@ -11257,6 +12300,11 @@
       </c>
       <c r="G179" s="3" t="inlineStr"/>
       <c r="H179" s="3" t="inlineStr"/>
+      <c r="I179" s="3" t="inlineStr"/>
+      <c r="J179" s="3" t="inlineStr"/>
+      <c r="K179" s="3" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr"/>
+      <c r="M179" s="3" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n">
@@ -11281,6 +12329,11 @@
       </c>
       <c r="G180" s="3" t="inlineStr"/>
       <c r="H180" s="3" t="inlineStr"/>
+      <c r="I180" s="3" t="inlineStr"/>
+      <c r="J180" s="3" t="inlineStr"/>
+      <c r="K180" s="3" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr"/>
+      <c r="M180" s="3" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n">
@@ -11305,6 +12358,11 @@
       </c>
       <c r="G181" s="3" t="inlineStr"/>
       <c r="H181" s="3" t="inlineStr"/>
+      <c r="I181" s="3" t="inlineStr"/>
+      <c r="J181" s="3" t="inlineStr"/>
+      <c r="K181" s="3" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr"/>
+      <c r="M181" s="3" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n">
@@ -11329,6 +12387,11 @@
       </c>
       <c r="G182" s="3" t="inlineStr"/>
       <c r="H182" s="3" t="inlineStr"/>
+      <c r="I182" s="3" t="inlineStr"/>
+      <c r="J182" s="3" t="inlineStr"/>
+      <c r="K182" s="3" t="inlineStr"/>
+      <c r="L182" s="3" t="inlineStr"/>
+      <c r="M182" s="3" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n">
@@ -11353,6 +12416,11 @@
       </c>
       <c r="G183" s="3" t="inlineStr"/>
       <c r="H183" s="3" t="inlineStr"/>
+      <c r="I183" s="3" t="inlineStr"/>
+      <c r="J183" s="3" t="inlineStr"/>
+      <c r="K183" s="3" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr"/>
+      <c r="M183" s="3" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n">
@@ -11377,6 +12445,11 @@
       </c>
       <c r="G184" s="3" t="inlineStr"/>
       <c r="H184" s="3" t="inlineStr"/>
+      <c r="I184" s="3" t="inlineStr"/>
+      <c r="J184" s="3" t="inlineStr"/>
+      <c r="K184" s="3" t="inlineStr"/>
+      <c r="L184" s="3" t="inlineStr"/>
+      <c r="M184" s="3" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n">
@@ -11401,6 +12474,11 @@
       </c>
       <c r="G185" s="3" t="inlineStr"/>
       <c r="H185" s="3" t="inlineStr"/>
+      <c r="I185" s="3" t="inlineStr"/>
+      <c r="J185" s="3" t="inlineStr"/>
+      <c r="K185" s="3" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr"/>
+      <c r="M185" s="3" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n">
@@ -11425,6 +12503,11 @@
       </c>
       <c r="G186" s="3" t="inlineStr"/>
       <c r="H186" s="3" t="inlineStr"/>
+      <c r="I186" s="3" t="inlineStr"/>
+      <c r="J186" s="3" t="inlineStr"/>
+      <c r="K186" s="3" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr"/>
+      <c r="M186" s="3" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n">
@@ -11449,6 +12532,11 @@
       </c>
       <c r="G187" s="3" t="inlineStr"/>
       <c r="H187" s="3" t="inlineStr"/>
+      <c r="I187" s="3" t="inlineStr"/>
+      <c r="J187" s="3" t="inlineStr"/>
+      <c r="K187" s="3" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr"/>
+      <c r="M187" s="3" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n">
@@ -11473,6 +12561,11 @@
       </c>
       <c r="G188" s="3" t="inlineStr"/>
       <c r="H188" s="3" t="inlineStr"/>
+      <c r="I188" s="3" t="inlineStr"/>
+      <c r="J188" s="3" t="inlineStr"/>
+      <c r="K188" s="3" t="inlineStr"/>
+      <c r="L188" s="3" t="inlineStr"/>
+      <c r="M188" s="3" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n">
@@ -11497,6 +12590,11 @@
       </c>
       <c r="G189" s="3" t="inlineStr"/>
       <c r="H189" s="3" t="inlineStr"/>
+      <c r="I189" s="3" t="inlineStr"/>
+      <c r="J189" s="3" t="inlineStr"/>
+      <c r="K189" s="3" t="inlineStr"/>
+      <c r="L189" s="3" t="inlineStr"/>
+      <c r="M189" s="3" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n">
@@ -11521,6 +12619,11 @@
       </c>
       <c r="G190" s="3" t="inlineStr"/>
       <c r="H190" s="3" t="inlineStr"/>
+      <c r="I190" s="3" t="inlineStr"/>
+      <c r="J190" s="3" t="inlineStr"/>
+      <c r="K190" s="3" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr"/>
+      <c r="M190" s="3" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n">
@@ -11545,6 +12648,11 @@
       </c>
       <c r="G191" s="3" t="inlineStr"/>
       <c r="H191" s="3" t="inlineStr"/>
+      <c r="I191" s="3" t="inlineStr"/>
+      <c r="J191" s="3" t="inlineStr"/>
+      <c r="K191" s="3" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr"/>
+      <c r="M191" s="3" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n">
@@ -11569,6 +12677,11 @@
       </c>
       <c r="G192" s="3" t="inlineStr"/>
       <c r="H192" s="3" t="inlineStr"/>
+      <c r="I192" s="3" t="inlineStr"/>
+      <c r="J192" s="3" t="inlineStr"/>
+      <c r="K192" s="3" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr"/>
+      <c r="M192" s="3" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n">
@@ -11593,6 +12706,11 @@
       </c>
       <c r="G193" s="3" t="inlineStr"/>
       <c r="H193" s="3" t="inlineStr"/>
+      <c r="I193" s="3" t="inlineStr"/>
+      <c r="J193" s="3" t="inlineStr"/>
+      <c r="K193" s="3" t="inlineStr"/>
+      <c r="L193" s="3" t="inlineStr"/>
+      <c r="M193" s="3" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n">
@@ -11617,6 +12735,11 @@
       </c>
       <c r="G194" s="3" t="inlineStr"/>
       <c r="H194" s="3" t="inlineStr"/>
+      <c r="I194" s="3" t="inlineStr"/>
+      <c r="J194" s="3" t="inlineStr"/>
+      <c r="K194" s="3" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr"/>
+      <c r="M194" s="3" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n">
@@ -11641,6 +12764,11 @@
       </c>
       <c r="G195" s="3" t="inlineStr"/>
       <c r="H195" s="3" t="inlineStr"/>
+      <c r="I195" s="3" t="inlineStr"/>
+      <c r="J195" s="3" t="inlineStr"/>
+      <c r="K195" s="3" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr"/>
+      <c r="M195" s="3" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n">
@@ -11665,6 +12793,11 @@
       </c>
       <c r="G196" s="3" t="inlineStr"/>
       <c r="H196" s="3" t="inlineStr"/>
+      <c r="I196" s="3" t="inlineStr"/>
+      <c r="J196" s="3" t="inlineStr"/>
+      <c r="K196" s="3" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr"/>
+      <c r="M196" s="3" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n">
@@ -11689,6 +12822,11 @@
       </c>
       <c r="G197" s="3" t="inlineStr"/>
       <c r="H197" s="3" t="inlineStr"/>
+      <c r="I197" s="3" t="inlineStr"/>
+      <c r="J197" s="3" t="inlineStr"/>
+      <c r="K197" s="3" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr"/>
+      <c r="M197" s="3" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n">
@@ -11713,6 +12851,11 @@
       </c>
       <c r="G198" s="3" t="inlineStr"/>
       <c r="H198" s="3" t="inlineStr"/>
+      <c r="I198" s="3" t="inlineStr"/>
+      <c r="J198" s="3" t="inlineStr"/>
+      <c r="K198" s="3" t="inlineStr"/>
+      <c r="L198" s="3" t="inlineStr"/>
+      <c r="M198" s="3" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n">
@@ -11737,6 +12880,11 @@
       </c>
       <c r="G199" s="3" t="inlineStr"/>
       <c r="H199" s="3" t="inlineStr"/>
+      <c r="I199" s="3" t="inlineStr"/>
+      <c r="J199" s="3" t="inlineStr"/>
+      <c r="K199" s="3" t="inlineStr"/>
+      <c r="L199" s="3" t="inlineStr"/>
+      <c r="M199" s="3" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="n">
@@ -11765,6 +12913,11 @@
       <c r="H200" s="3" t="n">
         <v>50</v>
       </c>
+      <c r="I200" s="3" t="inlineStr"/>
+      <c r="J200" s="3" t="inlineStr"/>
+      <c r="K200" s="3" t="inlineStr"/>
+      <c r="L200" s="3" t="inlineStr"/>
+      <c r="M200" s="3" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n">
@@ -11793,6 +12946,11 @@
       <c r="H201" s="3" t="n">
         <v>100</v>
       </c>
+      <c r="I201" s="3" t="inlineStr"/>
+      <c r="J201" s="3" t="inlineStr"/>
+      <c r="K201" s="3" t="inlineStr"/>
+      <c r="L201" s="3" t="inlineStr"/>
+      <c r="M201" s="3" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="n">
@@ -11821,6 +12979,11 @@
       <c r="H202" s="3" t="n">
         <v>150</v>
       </c>
+      <c r="I202" s="3" t="inlineStr"/>
+      <c r="J202" s="3" t="inlineStr"/>
+      <c r="K202" s="3" t="inlineStr"/>
+      <c r="L202" s="3" t="inlineStr"/>
+      <c r="M202" s="3" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n">
@@ -11849,6 +13012,11 @@
       <c r="H203" s="3" t="n">
         <v>200</v>
       </c>
+      <c r="I203" s="3" t="inlineStr"/>
+      <c r="J203" s="3" t="inlineStr"/>
+      <c r="K203" s="3" t="inlineStr"/>
+      <c r="L203" s="3" t="inlineStr"/>
+      <c r="M203" s="3" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n">
@@ -11877,6 +13045,11 @@
       <c r="H204" s="3" t="n">
         <v>250</v>
       </c>
+      <c r="I204" s="3" t="inlineStr"/>
+      <c r="J204" s="3" t="inlineStr"/>
+      <c r="K204" s="3" t="inlineStr"/>
+      <c r="L204" s="3" t="inlineStr"/>
+      <c r="M204" s="3" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n">
@@ -11905,6 +13078,11 @@
       <c r="H205" s="3" t="n">
         <v>300</v>
       </c>
+      <c r="I205" s="3" t="inlineStr"/>
+      <c r="J205" s="3" t="inlineStr"/>
+      <c r="K205" s="3" t="inlineStr"/>
+      <c r="L205" s="3" t="inlineStr"/>
+      <c r="M205" s="3" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n">
@@ -11933,6 +13111,11 @@
       <c r="H206" s="3" t="n">
         <v>350</v>
       </c>
+      <c r="I206" s="3" t="inlineStr"/>
+      <c r="J206" s="3" t="inlineStr"/>
+      <c r="K206" s="3" t="inlineStr"/>
+      <c r="L206" s="3" t="inlineStr"/>
+      <c r="M206" s="3" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n">
@@ -11961,6 +13144,11 @@
       <c r="H207" s="3" t="n">
         <v>400</v>
       </c>
+      <c r="I207" s="3" t="inlineStr"/>
+      <c r="J207" s="3" t="inlineStr"/>
+      <c r="K207" s="3" t="inlineStr"/>
+      <c r="L207" s="3" t="inlineStr"/>
+      <c r="M207" s="3" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n">
@@ -11989,6 +13177,11 @@
       <c r="H208" s="3" t="n">
         <v>450</v>
       </c>
+      <c r="I208" s="3" t="inlineStr"/>
+      <c r="J208" s="3" t="inlineStr"/>
+      <c r="K208" s="3" t="inlineStr"/>
+      <c r="L208" s="3" t="inlineStr"/>
+      <c r="M208" s="3" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n">
@@ -12017,6 +13210,11 @@
       <c r="H209" s="3" t="n">
         <v>500</v>
       </c>
+      <c r="I209" s="3" t="inlineStr"/>
+      <c r="J209" s="3" t="inlineStr"/>
+      <c r="K209" s="3" t="inlineStr"/>
+      <c r="L209" s="3" t="inlineStr"/>
+      <c r="M209" s="3" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n">
@@ -12045,6 +13243,11 @@
       <c r="H210" s="3" t="n">
         <v>550</v>
       </c>
+      <c r="I210" s="3" t="inlineStr"/>
+      <c r="J210" s="3" t="inlineStr"/>
+      <c r="K210" s="3" t="inlineStr"/>
+      <c r="L210" s="3" t="inlineStr"/>
+      <c r="M210" s="3" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n">
@@ -12073,6 +13276,11 @@
       <c r="H211" s="3" t="n">
         <v>600</v>
       </c>
+      <c r="I211" s="3" t="inlineStr"/>
+      <c r="J211" s="3" t="inlineStr"/>
+      <c r="K211" s="3" t="inlineStr"/>
+      <c r="L211" s="3" t="inlineStr"/>
+      <c r="M211" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12717,8 +13925,10 @@
       <c r="E2" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>1</v>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G2" s="3" t="n">
         <v>15</v>
@@ -12755,14 +13965,16 @@
       <c r="E3" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>1</v>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G3" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>1.89</v>
+        <v>1</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
@@ -12793,14 +14005,16 @@
       <c r="E4" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>1</v>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G4" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>1.78</v>
+        <v>1</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
@@ -12831,14 +14045,16 @@
       <c r="E5" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F5" s="3" t="n">
-        <v>1</v>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G5" s="3" t="n">
         <v>30</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>1.67</v>
+        <v>1</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
@@ -12869,14 +14085,16 @@
       <c r="E6" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F6" s="3" t="n">
-        <v>1</v>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G6" s="3" t="n">
         <v>35</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>1.56</v>
+        <v>1</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
@@ -12907,14 +14125,16 @@
       <c r="E7" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F7" s="3" t="n">
-        <v>1</v>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G7" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>1.45</v>
+        <v>1</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
@@ -12945,14 +14165,16 @@
       <c r="E8" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F8" s="3" t="n">
-        <v>1</v>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G8" s="3" t="n">
         <v>45</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>1.34</v>
+        <v>1</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
@@ -12983,14 +14205,16 @@
       <c r="E9" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F9" s="3" t="n">
-        <v>1</v>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G9" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>1.23</v>
+        <v>1</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
@@ -13021,14 +14245,16 @@
       <c r="E10" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F10" s="3" t="n">
-        <v>1</v>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G10" s="3" t="n">
         <v>55</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>1.12</v>
+        <v>1</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
@@ -13059,14 +14285,16 @@
       <c r="E11" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F11" s="3" t="n">
-        <v>1</v>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G11" s="3" t="n">
         <v>60</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
@@ -13097,14 +14325,16 @@
       <c r="E12" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F12" s="3" t="n">
-        <v>1</v>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G12" s="3" t="n">
         <v>65</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.91</v>
+        <v>0</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
@@ -13135,14 +14365,16 @@
       <c r="E13" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F13" s="3" t="n">
-        <v>1</v>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G13" s="3" t="n">
         <v>70</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
@@ -13173,14 +14405,16 @@
       <c r="E14" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F14" s="3" t="n">
-        <v>1</v>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G14" s="3" t="n">
         <v>75</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.71</v>
+        <v>0</v>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
@@ -13211,14 +14445,16 @@
       <c r="E15" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F15" s="3" t="n">
-        <v>1</v>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G15" s="3" t="n">
         <v>80</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.61</v>
+        <v>0</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
@@ -13249,14 +14485,16 @@
       <c r="E16" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F16" s="3" t="n">
-        <v>1</v>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G16" s="3" t="n">
         <v>85</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
@@ -13287,14 +14525,16 @@
       <c r="E17" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="F17" s="3" t="n">
-        <v>1</v>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G17" s="3" t="n">
         <v>90</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
@@ -13325,14 +14565,16 @@
       <c r="E18" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F18" s="3" t="n">
-        <v>1</v>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G18" s="3" t="n">
         <v>15</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
@@ -13363,14 +14605,16 @@
       <c r="E19" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F19" s="3" t="n">
-        <v>1</v>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G19" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>1.42</v>
+        <v>1</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
@@ -13401,14 +14645,16 @@
       <c r="E20" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F20" s="3" t="n">
-        <v>1</v>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G20" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>1.34</v>
+        <v>1</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
@@ -13439,14 +14685,16 @@
       <c r="E21" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F21" s="3" t="n">
-        <v>1</v>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G21" s="3" t="n">
         <v>30</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>1.26</v>
+        <v>1</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
@@ -13477,14 +14725,16 @@
       <c r="E22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F22" s="3" t="n">
-        <v>1</v>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G22" s="3" t="n">
         <v>35</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>1.18</v>
+        <v>1</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
@@ -13515,14 +14765,16 @@
       <c r="E23" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F23" s="3" t="n">
-        <v>1</v>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G23" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
@@ -13553,14 +14805,16 @@
       <c r="E24" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F24" s="3" t="n">
-        <v>1</v>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G24" s="3" t="n">
         <v>45</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
@@ -13591,14 +14845,16 @@
       <c r="E25" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F25" s="3" t="n">
-        <v>1</v>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G25" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
@@ -13629,14 +14885,16 @@
       <c r="E26" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F26" s="3" t="n">
-        <v>1</v>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G26" s="3" t="n">
         <v>55</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>0.86</v>
+        <v>0</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
@@ -13667,14 +14925,16 @@
       <c r="E27" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F27" s="3" t="n">
-        <v>1</v>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G27" s="3" t="n">
         <v>60</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0.78</v>
+        <v>0</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
@@ -13705,14 +14965,16 @@
       <c r="E28" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F28" s="3" t="n">
-        <v>1</v>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G28" s="3" t="n">
         <v>65</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
@@ -13743,14 +15005,16 @@
       <c r="E29" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F29" s="3" t="n">
-        <v>1</v>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G29" s="3" t="n">
         <v>70</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.62</v>
+        <v>0</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
@@ -13781,14 +15045,16 @@
       <c r="E30" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F30" s="3" t="n">
-        <v>1</v>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G30" s="3" t="n">
         <v>75</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>0.54</v>
+        <v>0</v>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
@@ -13819,14 +15085,16 @@
       <c r="E31" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F31" s="3" t="n">
-        <v>1</v>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G31" s="3" t="n">
         <v>80</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
@@ -13857,14 +15125,16 @@
       <c r="E32" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F32" s="3" t="n">
-        <v>1</v>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G32" s="3" t="n">
         <v>85</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0.38</v>
+        <v>0</v>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
@@ -13895,14 +15165,16 @@
       <c r="E33" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="F33" s="3" t="n">
-        <v>1</v>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G33" s="3" t="n">
         <v>90</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
@@ -13933,8 +15205,10 @@
       <c r="E34" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F34" s="3" t="n">
-        <v>1</v>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G34" s="3" t="n">
         <v>15</v>
@@ -13971,14 +15245,16 @@
       <c r="E35" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F35" s="3" t="n">
-        <v>1</v>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G35" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>2.82</v>
+        <v>2</v>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
@@ -14009,14 +15285,16 @@
       <c r="E36" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F36" s="3" t="n">
-        <v>1</v>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G36" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>2.64</v>
+        <v>2</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
@@ -14047,14 +15325,16 @@
       <c r="E37" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F37" s="3" t="n">
-        <v>1</v>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G37" s="3" t="n">
         <v>30</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>2.46</v>
+        <v>2</v>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
@@ -14085,14 +15365,16 @@
       <c r="E38" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F38" s="3" t="n">
-        <v>1</v>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G38" s="3" t="n">
         <v>35</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>2.28</v>
+        <v>2</v>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
@@ -14123,14 +15405,16 @@
       <c r="E39" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F39" s="3" t="n">
-        <v>1</v>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G39" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
@@ -14161,14 +15445,16 @@
       <c r="E40" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F40" s="3" t="n">
-        <v>1</v>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G40" s="3" t="n">
         <v>45</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>1.92</v>
+        <v>1</v>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
@@ -14199,14 +15485,16 @@
       <c r="E41" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F41" s="3" t="n">
-        <v>1</v>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G41" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>1.74</v>
+        <v>1</v>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
@@ -14237,14 +15525,16 @@
       <c r="E42" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F42" s="3" t="n">
-        <v>1</v>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G42" s="3" t="n">
         <v>55</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>1.56</v>
+        <v>1</v>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
@@ -14275,14 +15565,16 @@
       <c r="E43" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F43" s="3" t="n">
-        <v>1</v>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G43" s="3" t="n">
         <v>60</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>1.38</v>
+        <v>1</v>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
@@ -14313,14 +15605,16 @@
       <c r="E44" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F44" s="3" t="n">
-        <v>1</v>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G44" s="3" t="n">
         <v>65</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
@@ -14351,14 +15645,16 @@
       <c r="E45" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F45" s="3" t="n">
-        <v>1</v>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G45" s="3" t="n">
         <v>70</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
@@ -14389,14 +15685,16 @@
       <c r="E46" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F46" s="3" t="n">
-        <v>1</v>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G46" s="3" t="n">
         <v>75</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.84</v>
+        <v>0</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
@@ -14427,14 +15725,16 @@
       <c r="E47" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F47" s="3" t="n">
-        <v>1</v>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G47" s="3" t="n">
         <v>80</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>0.66</v>
+        <v>0</v>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
@@ -14465,14 +15765,16 @@
       <c r="E48" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F48" s="3" t="n">
-        <v>1</v>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G48" s="3" t="n">
         <v>85</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
@@ -14503,14 +15805,16 @@
       <c r="E49" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="F49" s="3" t="n">
-        <v>1</v>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G49" s="3" t="n">
         <v>90</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
@@ -14541,14 +15845,16 @@
       <c r="E50" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F50" s="3" t="n">
-        <v>1</v>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G50" s="3" t="n">
         <v>15</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
@@ -14579,14 +15885,16 @@
       <c r="E51" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F51" s="3" t="n">
-        <v>1</v>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G51" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>3.29</v>
+        <v>3</v>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
@@ -14617,14 +15925,16 @@
       <c r="E52" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F52" s="3" t="n">
-        <v>1</v>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G52" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>3.08</v>
+        <v>3</v>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
@@ -14655,14 +15965,16 @@
       <c r="E53" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F53" s="3" t="n">
-        <v>1</v>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G53" s="3" t="n">
         <v>30</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>2.87</v>
+        <v>2</v>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
@@ -14693,14 +16005,16 @@
       <c r="E54" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F54" s="3" t="n">
-        <v>1</v>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G54" s="3" t="n">
         <v>35</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>2.66</v>
+        <v>2</v>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
@@ -14731,14 +16045,16 @@
       <c r="E55" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F55" s="3" t="n">
-        <v>1</v>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G55" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>2.45</v>
+        <v>2</v>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
@@ -14769,14 +16085,16 @@
       <c r="E56" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F56" s="3" t="n">
-        <v>1</v>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G56" s="3" t="n">
         <v>45</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>2.24</v>
+        <v>2</v>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
@@ -14807,14 +16125,16 @@
       <c r="E57" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F57" s="3" t="n">
-        <v>1</v>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G57" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>2.03</v>
+        <v>2</v>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
@@ -14845,14 +16165,16 @@
       <c r="E58" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F58" s="3" t="n">
-        <v>1</v>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G58" s="3" t="n">
         <v>55</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>1.82</v>
+        <v>1</v>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
@@ -14883,14 +16205,16 @@
       <c r="E59" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F59" s="3" t="n">
-        <v>1</v>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G59" s="3" t="n">
         <v>60</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>1.61</v>
+        <v>1</v>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
@@ -14921,14 +16245,16 @@
       <c r="E60" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F60" s="3" t="n">
-        <v>1</v>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G60" s="3" t="n">
         <v>65</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
@@ -14959,14 +16285,16 @@
       <c r="E61" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F61" s="3" t="n">
-        <v>1</v>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G61" s="3" t="n">
         <v>70</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>1.19</v>
+        <v>1</v>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
@@ -14997,14 +16325,16 @@
       <c r="E62" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F62" s="3" t="n">
-        <v>1</v>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G62" s="3" t="n">
         <v>75</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>0.98</v>
+        <v>0</v>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
@@ -15035,14 +16365,16 @@
       <c r="E63" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F63" s="3" t="n">
-        <v>1</v>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G63" s="3" t="n">
         <v>80</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
@@ -15073,14 +16405,16 @@
       <c r="E64" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F64" s="3" t="n">
-        <v>1</v>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G64" s="3" t="n">
         <v>85</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0</v>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
@@ -15111,14 +16445,16 @@
       <c r="E65" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F65" s="3" t="n">
-        <v>1</v>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G65" s="3" t="n">
         <v>90</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
@@ -15149,8 +16485,10 @@
       <c r="E66" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F66" s="3" t="n">
-        <v>1</v>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G66" s="3" t="n">
         <v>15</v>
@@ -15187,14 +16525,16 @@
       <c r="E67" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F67" s="3" t="n">
-        <v>1</v>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G67" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>3.75</v>
+        <v>3</v>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
@@ -15225,14 +16565,16 @@
       <c r="E68" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F68" s="3" t="n">
-        <v>1</v>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G68" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
@@ -15263,14 +16605,16 @@
       <c r="E69" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F69" s="3" t="n">
-        <v>1</v>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G69" s="3" t="n">
         <v>30</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
@@ -15301,8 +16645,10 @@
       <c r="E70" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F70" s="3" t="n">
-        <v>1</v>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G70" s="3" t="n">
         <v>35</v>
@@ -15339,14 +16685,16 @@
       <c r="E71" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F71" s="3" t="n">
-        <v>1</v>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G71" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>2.75</v>
+        <v>2</v>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
@@ -15377,14 +16725,16 @@
       <c r="E72" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F72" s="3" t="n">
-        <v>1</v>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G72" s="3" t="n">
         <v>45</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
@@ -15415,14 +16765,16 @@
       <c r="E73" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F73" s="3" t="n">
-        <v>1</v>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G73" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>2.25</v>
+        <v>2</v>
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
@@ -15453,8 +16805,10 @@
       <c r="E74" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F74" s="3" t="n">
-        <v>1</v>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G74" s="3" t="n">
         <v>55</v>
@@ -15491,14 +16845,16 @@
       <c r="E75" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F75" s="3" t="n">
-        <v>1</v>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G75" s="3" t="n">
         <v>60</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>1.75</v>
+        <v>1</v>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
@@ -15529,14 +16885,16 @@
       <c r="E76" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F76" s="3" t="n">
-        <v>1</v>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G76" s="3" t="n">
         <v>65</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
@@ -15567,14 +16925,16 @@
       <c r="E77" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F77" s="3" t="n">
-        <v>1</v>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G77" s="3" t="n">
         <v>70</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="I77" s="3" t="inlineStr">
         <is>
@@ -15605,8 +16965,10 @@
       <c r="E78" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F78" s="3" t="n">
-        <v>1</v>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G78" s="3" t="n">
         <v>75</v>
@@ -15643,14 +17005,16 @@
       <c r="E79" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F79" s="3" t="n">
-        <v>1</v>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G79" s="3" t="n">
         <v>80</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="I79" s="3" t="inlineStr">
         <is>
@@ -15681,14 +17045,16 @@
       <c r="E80" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F80" s="3" t="n">
-        <v>1</v>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G80" s="3" t="n">
         <v>85</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I80" s="3" t="inlineStr">
         <is>
@@ -15719,14 +17085,16 @@
       <c r="E81" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F81" s="3" t="n">
-        <v>1</v>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G81" s="3" t="n">
         <v>90</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
@@ -15757,8 +17125,10 @@
       <c r="E82" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F82" s="3" t="n">
-        <v>1</v>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G82" s="3" t="n">
         <v>15</v>
@@ -15795,14 +17165,16 @@
       <c r="E83" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F83" s="3" t="n">
-        <v>1</v>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G83" s="3" t="n">
         <v>20</v>
       </c>
       <c r="H83" s="3" t="n">
-        <v>4.69</v>
+        <v>4</v>
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
@@ -15833,14 +17205,16 @@
       <c r="E84" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F84" s="3" t="n">
-        <v>1</v>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G84" s="3" t="n">
         <v>25</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>4.38</v>
+        <v>4</v>
       </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
@@ -15871,14 +17245,16 @@
       <c r="E85" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F85" s="3" t="n">
-        <v>1</v>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G85" s="3" t="n">
         <v>30</v>
       </c>
       <c r="H85" s="3" t="n">
-        <v>4.07</v>
+        <v>4</v>
       </c>
       <c r="I85" s="3" t="inlineStr">
         <is>
@@ -15909,14 +17285,16 @@
       <c r="E86" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F86" s="3" t="n">
-        <v>1</v>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G86" s="3" t="n">
         <v>35</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>3.76</v>
+        <v>3</v>
       </c>
       <c r="I86" s="3" t="inlineStr">
         <is>
@@ -15947,14 +17325,16 @@
       <c r="E87" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F87" s="3" t="n">
-        <v>1</v>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G87" s="3" t="n">
         <v>40</v>
       </c>
       <c r="H87" s="3" t="n">
-        <v>3.45</v>
+        <v>3</v>
       </c>
       <c r="I87" s="3" t="inlineStr">
         <is>
@@ -15985,14 +17365,16 @@
       <c r="E88" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F88" s="3" t="n">
-        <v>1</v>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G88" s="3" t="n">
         <v>45</v>
       </c>
       <c r="H88" s="3" t="n">
-        <v>3.14</v>
+        <v>3</v>
       </c>
       <c r="I88" s="3" t="inlineStr">
         <is>
@@ -16023,14 +17405,16 @@
       <c r="E89" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F89" s="3" t="n">
-        <v>1</v>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G89" s="3" t="n">
         <v>50</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>2.83</v>
+        <v>2</v>
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
@@ -16061,14 +17445,16 @@
       <c r="E90" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F90" s="3" t="n">
-        <v>1</v>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G90" s="3" t="n">
         <v>55</v>
       </c>
       <c r="H90" s="3" t="n">
-        <v>2.52</v>
+        <v>2</v>
       </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
@@ -16099,14 +17485,16 @@
       <c r="E91" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F91" s="3" t="n">
-        <v>1</v>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G91" s="3" t="n">
         <v>60</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>2.21</v>
+        <v>2</v>
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
@@ -16137,14 +17525,16 @@
       <c r="E92" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F92" s="3" t="n">
-        <v>1</v>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G92" s="3" t="n">
         <v>65</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>1.9</v>
+        <v>1</v>
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
@@ -16175,14 +17565,16 @@
       <c r="E93" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F93" s="3" t="n">
-        <v>1</v>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G93" s="3" t="n">
         <v>70</v>
       </c>
       <c r="H93" s="3" t="n">
-        <v>1.59</v>
+        <v>1</v>
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
@@ -16213,14 +17605,16 @@
       <c r="E94" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F94" s="3" t="n">
-        <v>1</v>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G94" s="3" t="n">
         <v>75</v>
       </c>
       <c r="H94" s="3" t="n">
-        <v>1.28</v>
+        <v>1</v>
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
@@ -16251,14 +17645,16 @@
       <c r="E95" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F95" s="3" t="n">
-        <v>1</v>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G95" s="3" t="n">
         <v>80</v>
       </c>
       <c r="H95" s="3" t="n">
-        <v>0.97</v>
+        <v>0</v>
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
@@ -16289,14 +17685,16 @@
       <c r="E96" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F96" s="3" t="n">
-        <v>1</v>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G96" s="3" t="n">
         <v>85</v>
       </c>
       <c r="H96" s="3" t="n">
-        <v>0.66</v>
+        <v>0</v>
       </c>
       <c r="I96" s="3" t="inlineStr">
         <is>
@@ -16327,14 +17725,16 @@
       <c r="E97" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="F97" s="3" t="n">
-        <v>1</v>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G97" s="3" t="n">
         <v>90</v>
       </c>
       <c r="H97" s="3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="I97" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix json_to_xlsx: format nested rewards, restore acupoint_rewards, sync item_pool from previous version
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/xlsx/items.xlsx
+++ b/config/xlsx/items.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_regular" sheetId="1" r:id="R62af063bf3534aa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_recipe_product" sheetId="2" r:id="Rdd09839da90245ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_effect" sheetId="3" r:id="R624f3985225f4816"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_launcher" sheetId="4" r:id="Rde922a2f72b54389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_crafting" sheetId="5" r:id="R57b1bace1b2e4580"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_regular" sheetId="1" r:id="Rbc761c76f6e343f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_recipe_product" sheetId="2" r:id="R49f47e4498a04d67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_effect" sheetId="3" r:id="R4ea6fe11db1a4b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_launcher" sheetId="4" r:id="R97f0e6f0d8934893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="items_crafting" sheetId="5" r:id="R173a7c84788b41e3"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>